<commit_message>
HAZOP node P&ID references, SIF-109 deviation
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013qGZUcwwWBAcAEPeh7Toud
</commit_message>
<xml_diff>
--- a/deliverables/06-wrapup/CFU-000-PM-EST-001_Cost-Estimate.xlsx
+++ b/deliverables/06-wrapup/CFU-000-PM-EST-001_Cost-Estimate.xlsx
@@ -455,7 +455,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>56731775.70104951</v>
+        <v>56791463.43148218</v>
       </c>
     </row>
     <row r="3">
@@ -465,7 +465,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>167817848.0389815</v>
+        <v>168016011.3040179</v>
       </c>
     </row>
     <row r="4">
@@ -475,7 +475,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>41954462.00974537</v>
+        <v>42004002.82600448</v>
       </c>
     </row>
     <row r="5">
@@ -485,7 +485,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>41954462.00974537</v>
+        <v>42004002.82600448</v>
       </c>
     </row>
     <row r="6">
@@ -495,7 +495,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>251726772.0584722</v>
+        <v>252024016.9560269</v>
       </c>
     </row>
     <row r="8">
@@ -505,7 +505,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>2517.267720584722</v>
+        <v>2520.240169560269</v>
       </c>
     </row>
   </sheetData>
@@ -519,7 +519,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G82"/>
+  <dimension ref="A1:G83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -2632,17 +2632,17 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>2 x 37 m3/h, 18.5 kW</t>
+          <t>2 x 37 m3/h, 30 kW</t>
         </is>
       </c>
       <c r="E68" t="n">
         <v>1</v>
       </c>
       <c r="F68" t="n">
-        <v>42348</v>
+        <v>49207</v>
       </c>
       <c r="G68" t="n">
-        <v>65162</v>
+        <v>75718</v>
       </c>
     </row>
     <row r="69">
@@ -2772,7 +2772,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>P-201A/B</t>
+          <t>P-119A/B</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -2782,28 +2782,28 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>LVGO pumparound / product</t>
+          <t>Flare KO drum pump-out</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>2 x 198 m3/h, 110 kW</t>
+          <t>2 x 21 m3/h, 7.5 kW</t>
         </is>
       </c>
       <c r="E73" t="n">
         <v>1</v>
       </c>
       <c r="F73" t="n">
-        <v>111439</v>
+        <v>31930</v>
       </c>
       <c r="G73" t="n">
-        <v>171477</v>
+        <v>49133</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>P-202A/B</t>
+          <t>P-201A/B</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -2813,28 +2813,28 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>HVGO pumparound / product</t>
+          <t>LVGO pumparound / product</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>2 x 391 m3/h, 200 kW</t>
+          <t>2 x 198 m3/h, 110 kW</t>
         </is>
       </c>
       <c r="E74" t="n">
-        <v>1.3</v>
+        <v>1</v>
       </c>
       <c r="F74" t="n">
-        <v>160933</v>
+        <v>111439</v>
       </c>
       <c r="G74" t="n">
-        <v>247635</v>
+        <v>171477</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>P-203A/B</t>
+          <t>P-202A/B</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -2844,28 +2844,28 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Slop wax</t>
+          <t>HVGO pumparound / product</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>2 x 12 m3/h, 5.5 kW</t>
+          <t>2 x 391 m3/h, 200 kW</t>
         </is>
       </c>
       <c r="E75" t="n">
         <v>1.3</v>
       </c>
       <c r="F75" t="n">
-        <v>35842</v>
+        <v>160933</v>
       </c>
       <c r="G75" t="n">
-        <v>55152</v>
+        <v>247635</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>P-204A/B</t>
+          <t>P-203A/B</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -2875,28 +2875,28 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Vacuum residue (incl. quench)</t>
+          <t>Slop wax</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>2 x 196 m3/h, 132 kW</t>
+          <t>2 x 12 m3/h, 5.5 kW</t>
         </is>
       </c>
       <c r="E76" t="n">
         <v>1.3</v>
       </c>
       <c r="F76" t="n">
-        <v>117955</v>
+        <v>35842</v>
       </c>
       <c r="G76" t="n">
-        <v>181504</v>
+        <v>55152</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>P-205A/B</t>
+          <t>P-204A/B</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -2906,28 +2906,28 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Hotwell sour water</t>
+          <t>Vacuum residue (incl. quench)</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>2 x 13 m3/h, 3.7 kW</t>
+          <t>2 x 196 m3/h, 132 kW</t>
         </is>
       </c>
       <c r="E77" t="n">
-        <v>1</v>
+        <v>1.3</v>
       </c>
       <c r="F77" t="n">
-        <v>26952</v>
+        <v>117955</v>
       </c>
       <c r="G77" t="n">
-        <v>41473</v>
+        <v>181504</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>P-206A/B</t>
+          <t>P-205A/B</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -2937,59 +2937,59 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Hotwell slop oil</t>
+          <t>Hotwell sour water</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>2 x 1 m3/h, 0.75 kW</t>
+          <t>2 x 13 m3/h, 3.7 kW</t>
         </is>
       </c>
       <c r="E78" t="n">
         <v>1</v>
       </c>
       <c r="F78" t="n">
-        <v>20402</v>
+        <v>26952</v>
       </c>
       <c r="G78" t="n">
-        <v>31393</v>
+        <v>41473</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>X-101</t>
+          <t>P-206A/B</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Package</t>
+          <t>Pump</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Demulsifier injection package</t>
+          <t>Hotwell slop oil</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>vendor package</t>
+          <t>2 x 1 m3/h, 0.75 kW</t>
         </is>
       </c>
       <c r="E79" t="n">
-        <v>1.3</v>
+        <v>1</v>
       </c>
       <c r="F79" t="n">
-        <v>120000</v>
+        <v>20402</v>
       </c>
       <c r="G79" t="n">
-        <v>184650</v>
+        <v>31393</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>X-102</t>
+          <t>X-101</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -2999,7 +2999,7 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Caustic injection package (desalted crude)</t>
+          <t>Demulsifier injection package</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -3020,7 +3020,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>X-103</t>
+          <t>X-102</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -3030,7 +3030,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Neutraliser / filming amine package (atm OH)</t>
+          <t>Caustic injection package (desalted crude)</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -3051,7 +3051,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>X-104</t>
+          <t>X-103</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -3061,7 +3061,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Corrosion inhibitor package (VDU OH)</t>
+          <t>Neutraliser / filming amine package (atm OH)</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -3076,6 +3076,37 @@
         <v>120000</v>
       </c>
       <c r="G82" t="n">
+        <v>184650</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>X-104</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Package</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>Corrosion inhibitor package (VDU OH)</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>vendor package</t>
+        </is>
+      </c>
+      <c r="E83" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="F83" t="n">
+        <v>120000</v>
+      </c>
+      <c r="G83" t="n">
         <v>184650</v>
       </c>
     </row>

</xml_diff>